<commit_message>
checkpoint: final state after DBx certification
</commit_message>
<xml_diff>
--- a/data/high_risk_qids.xlsx
+++ b/data/high_risk_qids.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dbx-study-app\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15C72497-0F2E-4711-BA5A-210C5EDADC33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F93A6A53-A4F9-4BC6-8B37-E149902A636B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="42">
   <si>
     <t>QID</t>
   </si>
@@ -1187,7 +1187,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>40</v>
       </c>
@@ -1210,7 +1210,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>39</v>
       </c>
@@ -1233,7 +1233,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>40</v>
       </c>
@@ -1256,7 +1256,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>40</v>
       </c>
@@ -1279,8 +1279,10 @@
         <v>21</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" s="6"/>
+    <row r="20" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="B20" s="6">
         <v>1373</v>
       </c>
@@ -1300,8 +1302,10 @@
         <v>23</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="6"/>
+    <row r="21" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="B21" s="6">
         <v>1897</v>
       </c>
@@ -1321,8 +1325,10 @@
         <v>23</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A22" s="6"/>
+    <row r="22" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="B22" s="6">
         <v>1127</v>
       </c>
@@ -1342,8 +1348,10 @@
         <v>23</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A23" s="6"/>
+    <row r="23" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="B23" s="6">
         <v>1783</v>
       </c>
@@ -1363,8 +1371,10 @@
         <v>24</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A24" s="6"/>
+    <row r="24" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="B24" s="6">
         <v>1821</v>
       </c>
@@ -1384,8 +1394,10 @@
         <v>25</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A25" s="6"/>
+    <row r="25" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="B25" s="6">
         <v>1219</v>
       </c>
@@ -1405,8 +1417,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A26" s="6"/>
+    <row r="26" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="B26" s="6">
         <v>1833</v>
       </c>
@@ -1426,8 +1440,10 @@
         <v>26</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A27" s="6"/>
+    <row r="27" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="B27" s="6">
         <v>1693</v>
       </c>
@@ -1447,8 +1463,10 @@
         <v>18</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A28" s="6"/>
+    <row r="28" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="B28" s="6">
         <v>1662</v>
       </c>
@@ -1468,8 +1486,10 @@
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A29" s="6"/>
+    <row r="29" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="B29" s="6">
         <v>1793</v>
       </c>
@@ -1489,8 +1509,10 @@
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A30" s="6"/>
+    <row r="30" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="B30" s="6">
         <v>1355</v>
       </c>
@@ -1510,8 +1532,10 @@
         <v>23</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A31" s="6"/>
+    <row r="31" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="B31" s="6">
         <v>1367</v>
       </c>
@@ -1531,8 +1555,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A32" s="6"/>
+    <row r="32" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="B32" s="6">
         <v>1477</v>
       </c>
@@ -1552,8 +1578,10 @@
         <v>23</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A33" s="6"/>
+    <row r="33" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="B33" s="6">
         <v>1277</v>
       </c>
@@ -1573,8 +1601,10 @@
         <v>29</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A34" s="6"/>
+    <row r="34" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="B34" s="6">
         <v>1861</v>
       </c>
@@ -1594,8 +1624,10 @@
         <v>30</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A35" s="6"/>
+    <row r="35" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="B35" s="6">
         <v>1863</v>
       </c>
@@ -1615,8 +1647,10 @@
         <v>32</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A36" s="6"/>
+    <row r="36" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="B36" s="6">
         <v>1325</v>
       </c>
@@ -1636,8 +1670,10 @@
         <v>23</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A37" s="6"/>
+    <row r="37" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="6" t="s">
+        <v>40</v>
+      </c>
       <c r="B37" s="6">
         <v>1479</v>
       </c>
@@ -1657,8 +1693,10 @@
         <v>23</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A38" s="6"/>
+    <row r="38" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="B38" s="6">
         <v>1297</v>
       </c>
@@ -1678,8 +1716,10 @@
         <v>23</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A39" s="6"/>
+    <row r="39" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="B39" s="6">
         <v>1456</v>
       </c>
@@ -1699,8 +1739,10 @@
         <v>10</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A40" s="6"/>
+    <row r="40" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="B40" s="6">
         <v>1827</v>
       </c>
@@ -1720,8 +1762,10 @@
         <v>24</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A41" s="6"/>
+    <row r="41" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="B41" s="6">
         <v>1381</v>
       </c>
@@ -1741,8 +1785,10 @@
         <v>23</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A42" s="6"/>
+    <row r="42" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="B42" s="6">
         <v>1713</v>
       </c>
@@ -1762,8 +1808,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A43" s="6"/>
+    <row r="43" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="B43" s="6">
         <v>1704</v>
       </c>
@@ -1783,8 +1831,10 @@
         <v>11</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A44" s="6"/>
+    <row r="44" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="B44" s="6">
         <v>1654</v>
       </c>
@@ -1804,8 +1854,10 @@
         <v>23</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A45" s="6"/>
+    <row r="45" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="6" t="s">
+        <v>40</v>
+      </c>
       <c r="B45" s="6">
         <v>1697</v>
       </c>
@@ -1825,8 +1877,10 @@
         <v>23</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A46" s="6"/>
+    <row r="46" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="B46" s="6">
         <v>1543</v>
       </c>
@@ -1846,8 +1900,10 @@
         <v>19</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A47" s="6"/>
+    <row r="47" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="B47" s="6">
         <v>1613</v>
       </c>
@@ -1867,8 +1923,10 @@
         <v>16</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A48" s="6"/>
+    <row r="48" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="6" t="s">
+        <v>40</v>
+      </c>
       <c r="B48" s="6">
         <v>1682</v>
       </c>
@@ -1888,8 +1946,10 @@
         <v>23</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A49" s="6"/>
+    <row r="49" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="B49" s="6">
         <v>1586</v>
       </c>
@@ -1909,8 +1969,10 @@
         <v>19</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A50" s="6"/>
+    <row r="50" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="B50" s="6">
         <v>1607</v>
       </c>

</xml_diff>